<commit_message>
Polish learner-facing copy, preserve kiosk navigation, and update WBS
</commit_message>
<xml_diff>
--- a/docs/CultureBridge_WBS_실제현황_2026-10-25.xlsx
+++ b/docs/CultureBridge_WBS_실제현황_2026-10-25.xlsx
@@ -2556,8 +2556,10 @@
       <c r="D4" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="7" t="s">
-        <v>20</v>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
+          <t>학습 서비스 목적 정하기</t>
+        </is>
       </c>
       <c r="F4" s="10" t="s">
         <v>21</v>
@@ -2628,8 +2630,10 @@
         <v>18</v>
       </c>
       <c r="D5" s="40"/>
-      <c r="E5" s="7" t="s">
-        <v>23</v>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>지원할 기능·제외할 기능</t>
+        </is>
       </c>
       <c r="F5" s="10" t="s">
         <v>21</v>
@@ -2702,8 +2706,10 @@
       <c r="D6" s="40" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="7" t="s">
-        <v>25</v>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>처음 배우는 과정 구성</t>
+        </is>
       </c>
       <c r="F6" s="10" t="s">
         <v>21</v>
@@ -2774,8 +2780,10 @@
         <v>18</v>
       </c>
       <c r="D7" s="40"/>
-      <c r="E7" s="7" t="s">
-        <v>26</v>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>관심 주제 탐구·복습 과정</t>
+        </is>
       </c>
       <c r="F7" s="10" t="s">
         <v>21</v>
@@ -2850,7 +2858,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>목표·성공 기준 설계</t>
+          <t>학습 목표·달성 기준</t>
         </is>
       </c>
       <c r="F8" s="10" t="s">
@@ -2924,7 +2932,7 @@
       <c r="D9" s="40"/>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>관찰·재계획·복구 설계</t>
+          <t>결과 확인·계획 수정·복구</t>
         </is>
       </c>
       <c r="F9" s="10" t="s">
@@ -2998,8 +3006,10 @@
       <c r="D10" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>31</v>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>검색·비교·코스 연결</t>
+        </is>
       </c>
       <c r="F10" s="10" t="s">
         <v>21</v>
@@ -3072,8 +3082,10 @@
       <c r="D11" s="40" t="s">
         <v>32</v>
       </c>
-      <c r="E11" s="7" t="s">
-        <v>33</v>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>관심사·목표의 우선순위</t>
+        </is>
       </c>
       <c r="F11" s="10" t="s">
         <v>21</v>
@@ -3144,8 +3156,10 @@
         <v>18</v>
       </c>
       <c r="D12" s="40"/>
-      <c r="E12" s="7" t="s">
-        <v>34</v>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>설명 방식·자세함 기준</t>
+        </is>
       </c>
       <c r="F12" s="10" t="s">
         <v>21</v>
@@ -3292,7 +3306,7 @@
       <c r="D14" s="40"/>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>주제 변경·이전 입력 분리</t>
+          <t>주제 변경·이전 질문 구분</t>
         </is>
       </c>
       <c r="F14" s="10" t="s">
@@ -3438,8 +3452,10 @@
         <v>18</v>
       </c>
       <c r="D16" s="40"/>
-      <c r="E16" s="7" t="s">
-        <v>40</v>
+      <c r="E16" s="7" t="inlineStr">
+        <is>
+          <t>개별 유산·사전 자료 범위</t>
+        </is>
       </c>
       <c r="F16" s="10" t="s">
         <v>21</v>
@@ -3658,8 +3674,10 @@
         <v>18</v>
       </c>
       <c r="D19" s="40"/>
-      <c r="E19" s="7" t="s">
-        <v>46</v>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>번역·AI 활용·배포 조건</t>
+        </is>
       </c>
       <c r="F19" s="10" t="s">
         <v>21</v>
@@ -3804,8 +3822,10 @@
         <v>18</v>
       </c>
       <c r="D21" s="40"/>
-      <c r="E21" s="7" t="s">
-        <v>49</v>
+      <c r="E21" s="7" t="inlineStr">
+        <is>
+          <t>음성 이용·전송 안내</t>
+        </is>
       </c>
       <c r="F21" s="10" t="s">
         <v>21</v>
@@ -3878,8 +3898,10 @@
       <c r="D22" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E22" s="7" t="s">
-        <v>51</v>
+      <c r="E22" s="7" t="inlineStr">
+        <is>
+          <t>웹·AI·저장 기술 선택</t>
+        </is>
       </c>
       <c r="F22" s="10" t="s">
         <v>21</v>
@@ -3952,8 +3974,10 @@
       <c r="D23" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="E23" s="7" t="s">
-        <v>53</v>
+      <c r="E23" s="7" t="inlineStr">
+        <is>
+          <t>담당·일정·완료 기준</t>
+        </is>
       </c>
       <c r="F23" s="10" t="s">
         <v>21</v>
@@ -4026,8 +4050,10 @@
       <c r="D24" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="E24" s="7" t="s">
-        <v>56</v>
+      <c r="E24" s="7" t="inlineStr">
+        <is>
+          <t>주요 메뉴·화면 나누기</t>
+        </is>
       </c>
       <c r="F24" s="10" t="s">
         <v>21</v>
@@ -4100,7 +4126,7 @@
       <c r="D25" s="40"/>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>중복 메뉴·검색 복귀 경로</t>
+          <t>겹친 메뉴·검색 복귀 경로</t>
         </is>
       </c>
       <c r="F25" s="10" t="s">
@@ -4246,8 +4272,10 @@
         <v>54</v>
       </c>
       <c r="D27" s="40"/>
-      <c r="E27" s="7" t="s">
-        <v>60</v>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>버튼·입력칸·카드 상태</t>
+        </is>
       </c>
       <c r="F27" s="10" t="s">
         <v>21</v>
@@ -4392,8 +4420,10 @@
         <v>54</v>
       </c>
       <c r="D29" s="40"/>
-      <c r="E29" s="7" t="s">
-        <v>63</v>
+      <c r="E29" s="7" t="inlineStr">
+        <is>
+          <t>자유 질문 시작 화면</t>
+        </is>
       </c>
       <c r="F29" s="10" t="s">
         <v>21</v>
@@ -4464,8 +4494,10 @@
         <v>54</v>
       </c>
       <c r="D30" s="40"/>
-      <c r="E30" s="7" t="s">
-        <v>64</v>
+      <c r="E30" s="7" t="inlineStr">
+        <is>
+          <t>유산 검색 시작 화면</t>
+        </is>
       </c>
       <c r="F30" s="10" t="s">
         <v>21</v>
@@ -4610,8 +4642,10 @@
         <v>54</v>
       </c>
       <c r="D32" s="40"/>
-      <c r="E32" s="7" t="s">
-        <v>67</v>
+      <c r="E32" s="7" t="inlineStr">
+        <is>
+          <t>대화 목록·기록 없음 안내</t>
+        </is>
       </c>
       <c r="F32" s="10" t="s">
         <v>21</v>
@@ -4686,7 +4720,7 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>발화·대화 퀴즈 배치</t>
+          <t>대화 내용·퀴즈 배치</t>
         </is>
       </c>
       <c r="F33" s="10" t="s">
@@ -4760,7 +4794,7 @@
       <c r="D34" s="40"/>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>근거·실행 과정 배치</t>
+          <t>출처·진행 과정 배치</t>
         </is>
       </c>
       <c r="F34" s="10" t="s">
@@ -4906,8 +4940,10 @@
         <v>54</v>
       </c>
       <c r="D36" s="40"/>
-      <c r="E36" s="7" t="s">
-        <v>73</v>
+      <c r="E36" s="7" t="inlineStr">
+        <is>
+          <t>관심사·목표 관리 화면</t>
+        </is>
       </c>
       <c r="F36" s="10" t="s">
         <v>21</v>
@@ -5052,8 +5088,10 @@
       <c r="D38" s="40" t="s">
         <v>75</v>
       </c>
-      <c r="E38" s="7" t="s">
-        <v>76</v>
+      <c r="E38" s="7" t="inlineStr">
+        <is>
+          <t>검색 입력칸·결과 카드</t>
+        </is>
       </c>
       <c r="F38" s="10" t="s">
         <v>21</v>
@@ -5126,7 +5164,7 @@
       <c r="D39" s="40"/>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>빈 결과·공식 원문 안내</t>
+          <t>검색 결과 없음·원문 안내</t>
         </is>
       </c>
       <c r="F39" s="10" t="s">
@@ -5200,8 +5238,10 @@
       <c r="D40" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="E40" s="7" t="s">
-        <v>79</v>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>한글·영어 검색어 제안</t>
+        </is>
       </c>
       <c r="F40" s="10" t="s">
         <v>21</v>
@@ -5490,8 +5530,10 @@
         <v>54</v>
       </c>
       <c r="D44" s="40"/>
-      <c r="E44" s="7" t="s">
-        <v>84</v>
+      <c r="E44" s="7" t="inlineStr">
+        <is>
+          <t>비교 학습으로 이동</t>
+        </is>
       </c>
       <c r="F44" s="10" t="s">
         <v>21</v>
@@ -5564,8 +5606,10 @@
       <c r="D45" s="40" t="s">
         <v>85</v>
       </c>
-      <c r="E45" s="7" t="s">
-        <v>86</v>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>국내외 구분·추천 이유</t>
+        </is>
       </c>
       <c r="F45" s="10" t="s">
         <v>21</v>
@@ -5636,8 +5680,10 @@
         <v>54</v>
       </c>
       <c r="D46" s="40"/>
-      <c r="E46" s="7" t="s">
-        <v>87</v>
+      <c r="E46" s="7" t="inlineStr">
+        <is>
+          <t>후보가 적을 때 안내</t>
+        </is>
       </c>
       <c r="F46" s="10" t="s">
         <v>21</v>
@@ -5784,7 +5830,7 @@
       <c r="D48" s="40"/>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>근거·질문·학습 단계</t>
+          <t>출처·질문·학습 순서</t>
         </is>
       </c>
       <c r="F48" s="10" t="s">
@@ -5858,8 +5904,10 @@
       <c r="D49" s="40" t="s">
         <v>91</v>
       </c>
-      <c r="E49" s="7" t="s">
-        <v>92</v>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>문제·보기·제출 배치</t>
+        </is>
       </c>
       <c r="F49" s="10" t="s">
         <v>21</v>
@@ -5930,8 +5978,10 @@
         <v>54</v>
       </c>
       <c r="D50" s="40"/>
-      <c r="E50" s="7" t="s">
-        <v>93</v>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>채점·해설·복습으로 이동</t>
+        </is>
       </c>
       <c r="F50" s="10" t="s">
         <v>21</v>
@@ -6078,7 +6128,7 @@
       <c r="D52" s="40"/>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>목표·수준·시작 동선</t>
+          <t>목표·수준·시작 방법</t>
         </is>
       </c>
       <c r="F52" s="10" t="s">
@@ -6152,8 +6202,10 @@
       <c r="D53" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="E53" s="7" t="s">
-        <v>98</v>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>점수·오답·다시 학습하기</t>
+        </is>
       </c>
       <c r="F53" s="10" t="s">
         <v>21</v>
@@ -6224,8 +6276,10 @@
         <v>54</v>
       </c>
       <c r="D54" s="40"/>
-      <c r="E54" s="7" t="s">
-        <v>99</v>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>비교 기록·활동지 보기</t>
+        </is>
       </c>
       <c r="F54" s="10" t="s">
         <v>21</v>
@@ -6444,8 +6498,10 @@
       <c r="D57" s="40" t="s">
         <v>103</v>
       </c>
-      <c r="E57" s="7" t="s">
-        <v>104</v>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>화면 크기·터치·초점 배치</t>
+        </is>
       </c>
       <c r="F57" s="10" t="s">
         <v>21</v>
@@ -6516,8 +6572,10 @@
         <v>54</v>
       </c>
       <c r="D58" s="40"/>
-      <c r="E58" s="7" t="s">
-        <v>105</v>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>체험 화면 초기화 과정</t>
+        </is>
       </c>
       <c r="F58" s="10" t="s">
         <v>21</v>
@@ -6592,7 +6650,7 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>목표·자료·대기 요청 구조</t>
+          <t>목표·자료·대기 요청 구성</t>
         </is>
       </c>
       <c r="F59" s="10" t="s">
@@ -6664,8 +6722,10 @@
         <v>106</v>
       </c>
       <c r="D60" s="40"/>
-      <c r="E60" s="7" t="s">
-        <v>109</v>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>대화 수정 번호·중단 상태</t>
+        </is>
       </c>
       <c r="F60" s="10" t="s">
         <v>21</v>
@@ -6738,8 +6798,10 @@
       <c r="D61" s="40" t="s">
         <v>110</v>
       </c>
-      <c r="E61" s="7" t="s">
-        <v>111</v>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>학습 개념·직접 설명하기</t>
+        </is>
       </c>
       <c r="F61" s="10" t="s">
         <v>21</v>
@@ -6886,8 +6948,10 @@
       <c r="D63" s="40" t="s">
         <v>113</v>
       </c>
-      <c r="E63" s="7" t="s">
-        <v>114</v>
+      <c r="E63" s="7" t="inlineStr">
+        <is>
+          <t>예제·공식 자료 구별</t>
+        </is>
       </c>
       <c r="F63" s="10" t="s">
         <v>21</v>
@@ -6958,8 +7022,10 @@
         <v>106</v>
       </c>
       <c r="D64" s="40"/>
-      <c r="E64" s="7" t="s">
-        <v>115</v>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>개별·유산군·다른 이름</t>
+        </is>
       </c>
       <c r="F64" s="10" t="s">
         <v>21</v>
@@ -7034,7 +7100,7 @@
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>학습·답안 제출 규격</t>
+          <t>학습·답안 제출 방식</t>
         </is>
       </c>
       <c r="F65" s="10" t="s">
@@ -7106,8 +7172,10 @@
         <v>106</v>
       </c>
       <c r="D66" s="40"/>
-      <c r="E66" s="7" t="s">
-        <v>118</v>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>기록·설정 접근 기준</t>
+        </is>
       </c>
       <c r="F66" s="10" t="s">
         <v>21</v>
@@ -7180,8 +7248,10 @@
       <c r="D67" s="40" t="s">
         <v>119</v>
       </c>
-      <c r="E67" s="7" t="s">
-        <v>120</v>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>시간·호출 횟수·다시 시도</t>
+        </is>
       </c>
       <c r="F67" s="10" t="s">
         <v>21</v>
@@ -7254,7 +7324,7 @@
       <c r="D68" s="40"/>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>중복 요청·결과 재사용</t>
+          <t>중복 요청·이전 결과 활용</t>
         </is>
       </c>
       <c r="F68" s="10" t="s">
@@ -7402,8 +7472,10 @@
         <v>106</v>
       </c>
       <c r="D70" s="40"/>
-      <c r="E70" s="7" t="s">
-        <v>125</v>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>검색 목록·페이지 나누기</t>
+        </is>
       </c>
       <c r="F70" s="10" t="s">
         <v>21</v>
@@ -7548,8 +7620,10 @@
         <v>106</v>
       </c>
       <c r="D72" s="40"/>
-      <c r="E72" s="7" t="s">
-        <v>128</v>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>유산 번호·공식 출처 연결</t>
+        </is>
       </c>
       <c r="F72" s="10" t="s">
         <v>21</v>
@@ -7622,8 +7696,10 @@
       <c r="D73" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="E73" s="7" t="s">
-        <v>130</v>
+      <c r="E73" s="7" t="inlineStr">
+        <is>
+          <t>공식 위치·좌표 기준 구분</t>
+        </is>
       </c>
       <c r="F73" s="10" t="s">
         <v>21</v>
@@ -7696,8 +7772,10 @@
       <c r="D74" s="40" t="s">
         <v>131</v>
       </c>
-      <c r="E74" s="7" t="s">
-        <v>132</v>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>세계유산 목록 자동 수집</t>
+        </is>
       </c>
       <c r="F74" s="10" t="s">
         <v>21</v>
@@ -7768,8 +7846,10 @@
         <v>106</v>
       </c>
       <c r="D75" s="40"/>
-      <c r="E75" s="7" t="s">
-        <v>133</v>
+      <c r="E75" s="7" t="inlineStr">
+        <is>
+          <t>수동 파일·보관 자료 활용</t>
+        </is>
       </c>
       <c r="F75" s="10" t="s">
         <v>21</v>
@@ -7914,8 +7994,10 @@
         <v>106</v>
       </c>
       <c r="D77" s="40"/>
-      <c r="E77" s="7" t="s">
-        <v>136</v>
+      <c r="E77" s="7" t="inlineStr">
+        <is>
+          <t>개별 건물·유산 묶음 연결</t>
+        </is>
       </c>
       <c r="F77" s="10" t="s">
         <v>21</v>
@@ -7988,8 +8070,10 @@
       <c r="D78" s="40" t="s">
         <v>137</v>
       </c>
-      <c r="E78" s="7" t="s">
-        <v>138</v>
+      <c r="E78" s="7" t="inlineStr">
+        <is>
+          <t>한글·영어·다른 이름 검색</t>
+        </is>
       </c>
       <c r="F78" s="10" t="s">
         <v>21</v>
@@ -8134,8 +8218,10 @@
       <c r="D80" s="40" t="s">
         <v>140</v>
       </c>
-      <c r="E80" s="7" t="s">
-        <v>141</v>
+      <c r="E80" s="7" t="inlineStr">
+        <is>
+          <t>해당 유산·주변 유산 구별</t>
+        </is>
       </c>
       <c r="F80" s="10" t="s">
         <v>21</v>
@@ -8206,8 +8292,10 @@
         <v>106</v>
       </c>
       <c r="D81" s="40"/>
-      <c r="E81" s="7" t="s">
-        <v>142</v>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>개별 유산·유산 묶음 구분</t>
+        </is>
       </c>
       <c r="F81" s="10" t="s">
         <v>21</v>
@@ -8280,8 +8368,10 @@
       <c r="D82" s="40" t="s">
         <v>143</v>
       </c>
-      <c r="E82" s="7" t="s">
-        <v>144</v>
+      <c r="E82" s="7" t="inlineStr">
+        <is>
+          <t>보관 자료 갱신·만료 처리</t>
+        </is>
       </c>
       <c r="F82" s="10" t="s">
         <v>21</v>
@@ -8352,8 +8442,10 @@
         <v>106</v>
       </c>
       <c r="D83" s="40"/>
-      <c r="E83" s="7" t="s">
-        <v>145</v>
+      <c r="E83" s="7" t="inlineStr">
+        <is>
+          <t>자료 수집 실패 시 대안</t>
+        </is>
       </c>
       <c r="F83" s="10" t="s">
         <v>21</v>
@@ -8426,8 +8518,10 @@
       <c r="D84" s="40" t="s">
         <v>146</v>
       </c>
-      <c r="E84" s="7" t="s">
-        <v>147</v>
+      <c r="E84" s="7" t="inlineStr">
+        <is>
+          <t>자료 표시·저장 허용 범위</t>
+        </is>
       </c>
       <c r="F84" s="10" t="s">
         <v>21</v>
@@ -8498,8 +8592,10 @@
         <v>106</v>
       </c>
       <c r="D85" s="40"/>
-      <c r="E85" s="7" t="s">
-        <v>148</v>
+      <c r="E85" s="7" t="inlineStr">
+        <is>
+          <t>번역·AI 활용 허용 범위</t>
+        </is>
       </c>
       <c r="F85" s="10" t="s">
         <v>21</v>
@@ -8572,8 +8668,10 @@
       <c r="D86" s="40" t="s">
         <v>149</v>
       </c>
-      <c r="E86" s="7" t="s">
-        <v>150</v>
+      <c r="E86" s="7" t="inlineStr">
+        <is>
+          <t>단어·뜻풀이 찾기</t>
+        </is>
       </c>
       <c r="F86" s="10" t="s">
         <v>21</v>
@@ -8644,8 +8742,10 @@
         <v>106</v>
       </c>
       <c r="D87" s="40"/>
-      <c r="E87" s="7" t="s">
-        <v>151</v>
+      <c r="E87" s="7" t="inlineStr">
+        <is>
+          <t>출처·이용 조건 표시</t>
+        </is>
       </c>
       <c r="F87" s="10" t="s">
         <v>21</v>
@@ -8718,8 +8818,10 @@
       <c r="D88" s="40" t="s">
         <v>152</v>
       </c>
-      <c r="E88" s="7" t="s">
-        <v>153</v>
+      <c r="E88" s="7" t="inlineStr">
+        <is>
+          <t>실제 키·연결 응답 확인</t>
+        </is>
       </c>
       <c r="F88" s="10" t="s">
         <v>21</v>
@@ -8790,8 +8892,10 @@
         <v>18</v>
       </c>
       <c r="D89" s="40"/>
-      <c r="E89" s="7" t="s">
-        <v>154</v>
+      <c r="E89" s="7" t="inlineStr">
+        <is>
+          <t>호출 한도·키 오류 안내</t>
+        </is>
       </c>
       <c r="F89" s="10" t="s">
         <v>21</v>
@@ -8864,8 +8968,10 @@
       <c r="D90" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="E90" s="7" t="s">
-        <v>156</v>
+      <c r="E90" s="7" t="inlineStr">
+        <is>
+          <t>공개 자료·인증 범위 확인</t>
+        </is>
       </c>
       <c r="F90" s="10" t="s">
         <v>21</v>
@@ -9012,8 +9118,10 @@
       <c r="D92" s="40" t="s">
         <v>159</v>
       </c>
-      <c r="E92" s="7" t="s">
-        <v>160</v>
+      <c r="E92" s="7" t="inlineStr">
+        <is>
+          <t>서비스명·주요 메뉴 표시</t>
+        </is>
       </c>
       <c r="F92" s="10" t="s">
         <v>21</v>
@@ -9156,8 +9264,10 @@
         <v>54</v>
       </c>
       <c r="D94" s="40"/>
-      <c r="E94" s="7" t="s">
-        <v>162</v>
+      <c r="E94" s="7" t="inlineStr">
+        <is>
+          <t>하단 안내·설정으로 이동</t>
+        </is>
       </c>
       <c r="F94" s="10" t="s">
         <v>21</v>
@@ -9302,8 +9412,10 @@
         <v>54</v>
       </c>
       <c r="D96" s="40"/>
-      <c r="E96" s="7" t="s">
-        <v>165</v>
+      <c r="E96" s="7" t="inlineStr">
+        <is>
+          <t>버튼·입력칸·펼치기 통일</t>
+        </is>
       </c>
       <c r="F96" s="10" t="s">
         <v>21</v>
@@ -9448,8 +9560,10 @@
         <v>54</v>
       </c>
       <c r="D98" s="40"/>
-      <c r="E98" s="7" t="s">
-        <v>168</v>
+      <c r="E98" s="7" t="inlineStr">
+        <is>
+          <t>역사 대화 시작하기</t>
+        </is>
       </c>
       <c r="F98" s="10" t="s">
         <v>21</v>
@@ -9520,8 +9634,10 @@
         <v>54</v>
       </c>
       <c r="D99" s="40"/>
-      <c r="E99" s="7" t="s">
-        <v>169</v>
+      <c r="E99" s="7" t="inlineStr">
+        <is>
+          <t>유산 탐구 시작하기</t>
+        </is>
       </c>
       <c r="F99" s="10" t="s">
         <v>21</v>
@@ -9670,7 +9786,7 @@
       <c r="D101" s="40"/>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>실행 과정·중단 안내</t>
+          <t>진행 과정·중단 안내</t>
         </is>
       </c>
       <c r="F101" s="10" t="s">
@@ -9746,7 +9862,7 @@
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>대화 목록·이어가기 동선</t>
+          <t>대화 목록·이어가기 이동</t>
         </is>
       </c>
       <c r="F102" s="10" t="s">
@@ -9818,8 +9934,10 @@
         <v>54</v>
       </c>
       <c r="D103" s="40"/>
-      <c r="E103" s="7" t="s">
-        <v>175</v>
+      <c r="E103" s="7" t="inlineStr">
+        <is>
+          <t>대화 기록 없음 안내</t>
+        </is>
       </c>
       <c r="F103" s="10" t="s">
         <v>21</v>
@@ -9894,7 +10012,7 @@
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>발화·계획·학습 관찰 표시</t>
+          <t>대화·계획·학습 변화 표시</t>
         </is>
       </c>
       <c r="F104" s="10" t="s">
@@ -10188,7 +10306,7 @@
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>설명 문체·적용 범위</t>
+          <t>설명 방식·적용 범위</t>
         </is>
       </c>
       <c r="F108" s="10" t="s">
@@ -10260,8 +10378,10 @@
         <v>54</v>
       </c>
       <c r="D109" s="40"/>
-      <c r="E109" s="7" t="s">
-        <v>183</v>
+      <c r="E109" s="7" t="inlineStr">
+        <is>
+          <t>설명 설정 저장·불러오기</t>
+        </is>
       </c>
       <c r="F109" s="10" t="s">
         <v>21</v>
@@ -10334,8 +10454,10 @@
       <c r="D110" s="40" t="s">
         <v>184</v>
       </c>
-      <c r="E110" s="7" t="s">
-        <v>185</v>
+      <c r="E110" s="7" t="inlineStr">
+        <is>
+          <t>파악한 관심사·목표 요약</t>
+        </is>
       </c>
       <c r="F110" s="10" t="s">
         <v>21</v>
@@ -10552,8 +10674,10 @@
       <c r="D113" s="40" t="s">
         <v>188</v>
       </c>
-      <c r="E113" s="7" t="s">
-        <v>189</v>
+      <c r="E113" s="7" t="inlineStr">
+        <is>
+          <t>음성 입력 시작·중단</t>
+        </is>
       </c>
       <c r="F113" s="10" t="s">
         <v>21</v>
@@ -10624,8 +10748,10 @@
         <v>54</v>
       </c>
       <c r="D114" s="40"/>
-      <c r="E114" s="7" t="s">
-        <v>190</v>
+      <c r="E114" s="7" t="inlineStr">
+        <is>
+          <t>글자로 바뀐 음성 확인</t>
+        </is>
       </c>
       <c r="F114" s="10" t="s">
         <v>21</v>
@@ -10914,8 +11040,10 @@
         <v>54</v>
       </c>
       <c r="D118" s="40"/>
-      <c r="E118" s="7" t="s">
-        <v>195</v>
+      <c r="E118" s="7" t="inlineStr">
+        <is>
+          <t>목록·페이지·검색 조건 유지</t>
+        </is>
       </c>
       <c r="F118" s="10" t="s">
         <v>21</v>
@@ -11136,8 +11264,10 @@
       <c r="D121" s="40" t="s">
         <v>199</v>
       </c>
-      <c r="E121" s="7" t="s">
-        <v>200</v>
+      <c r="E121" s="7" t="inlineStr">
+        <is>
+          <t>한글·영어·국가명 검색</t>
+        </is>
       </c>
       <c r="F121" s="10" t="s">
         <v>21</v>
@@ -11498,8 +11628,10 @@
         <v>54</v>
       </c>
       <c r="D126" s="40"/>
-      <c r="E126" s="7" t="s">
-        <v>206</v>
+      <c r="E126" s="7" t="inlineStr">
+        <is>
+          <t>비교 탐구로 이동</t>
+        </is>
       </c>
       <c r="F126" s="10" t="s">
         <v>21</v>
@@ -11644,8 +11776,10 @@
         <v>54</v>
       </c>
       <c r="D128" s="40"/>
-      <c r="E128" s="7" t="s">
-        <v>209</v>
+      <c r="E128" s="7" t="inlineStr">
+        <is>
+          <t>비교 시작·판단 보류 안내</t>
+        </is>
       </c>
       <c r="F128" s="10" t="s">
         <v>21</v>
@@ -11864,7 +11998,7 @@
       <c r="D131" s="40"/>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>질문 인용·의미 대조</t>
+          <t>답변 근거·질문 뜻 확인</t>
         </is>
       </c>
       <c r="F131" s="10" t="s">
@@ -11938,8 +12072,10 @@
       <c r="D132" s="40" t="s">
         <v>214</v>
       </c>
-      <c r="E132" s="7" t="s">
-        <v>215</v>
+      <c r="E132" s="7" t="inlineStr">
+        <is>
+          <t>답안 선택·제출 처리</t>
+        </is>
       </c>
       <c r="F132" s="10" t="s">
         <v>21</v>
@@ -12084,8 +12220,10 @@
         <v>54</v>
       </c>
       <c r="D134" s="40"/>
-      <c r="E134" s="7" t="s">
-        <v>217</v>
+      <c r="E134" s="7" t="inlineStr">
+        <is>
+          <t>오답 복습으로 이동</t>
+        </is>
       </c>
       <c r="F134" s="10" t="s">
         <v>21</v>
@@ -12306,7 +12444,7 @@
       <c r="D137" s="40"/>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>수준 선택·상단 시작 버튼</t>
+          <t>수준 선택·학습 시작 버튼</t>
         </is>
       </c>
       <c r="F137" s="10" t="s">
@@ -12452,8 +12590,10 @@
         <v>54</v>
       </c>
       <c r="D139" s="40"/>
-      <c r="E139" s="7" t="s">
-        <v>224</v>
+      <c r="E139" s="7" t="inlineStr">
+        <is>
+          <t>저장 비교·다시 탐구하기</t>
+        </is>
       </c>
       <c r="F139" s="10" t="s">
         <v>21</v>
@@ -12524,8 +12664,10 @@
         <v>54</v>
       </c>
       <c r="D140" s="40"/>
-      <c r="E140" s="7" t="s">
-        <v>225</v>
+      <c r="E140" s="7" t="inlineStr">
+        <is>
+          <t>학습 결과 인쇄하기</t>
+        </is>
       </c>
       <c r="F140" s="10" t="s">
         <v>21</v>
@@ -12746,8 +12888,10 @@
       <c r="D143" s="40" t="s">
         <v>229</v>
       </c>
-      <c r="E143" s="7" t="s">
-        <v>230</v>
+      <c r="E143" s="7" t="inlineStr">
+        <is>
+          <t>홈 화면 추가·업데이트</t>
+        </is>
       </c>
       <c r="F143" s="10" t="s">
         <v>21</v>
@@ -12818,8 +12962,10 @@
         <v>54</v>
       </c>
       <c r="D144" s="40"/>
-      <c r="E144" s="7" t="s">
-        <v>231</v>
+      <c r="E144" s="7" t="inlineStr">
+        <is>
+          <t>인터넷 연결 끊김 안내</t>
+        </is>
       </c>
       <c r="F144" s="10" t="s">
         <v>21</v>
@@ -13038,8 +13184,10 @@
       <c r="D147" s="40" t="s">
         <v>235</v>
       </c>
-      <c r="E147" s="7" t="s">
-        <v>236</v>
+      <c r="E147" s="7" t="inlineStr">
+        <is>
+          <t>휴대전화 배치·본문 너비</t>
+        </is>
       </c>
       <c r="F147" s="10" t="s">
         <v>21</v>
@@ -13110,8 +13258,10 @@
         <v>54</v>
       </c>
       <c r="D148" s="40"/>
-      <c r="E148" s="7" t="s">
-        <v>237</v>
+      <c r="E148" s="7" t="inlineStr">
+        <is>
+          <t>초점·터치·화면 움직임 줄임</t>
+        </is>
       </c>
       <c r="F148" s="10" t="s">
         <v>21</v>
@@ -13184,8 +13334,10 @@
       <c r="D149" s="40" t="s">
         <v>238</v>
       </c>
-      <c r="E149" s="7" t="s">
-        <v>239</v>
+      <c r="E149" s="7" t="inlineStr">
+        <is>
+          <t>비밀 키·AI 모델 설정</t>
+        </is>
       </c>
       <c r="F149" s="10" t="s">
         <v>21</v>
@@ -13256,8 +13408,10 @@
         <v>106</v>
       </c>
       <c r="D150" s="40"/>
-      <c r="E150" s="7" t="s">
-        <v>240</v>
+      <c r="E150" s="7" t="inlineStr">
+        <is>
+          <t>응답 형식·시간 제한</t>
+        </is>
       </c>
       <c r="F150" s="10" t="s">
         <v>21</v>
@@ -13332,7 +13486,7 @@
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>계획·도구·관찰 연결</t>
+          <t>AI 계획·도구·결과 연결</t>
         </is>
       </c>
       <c r="F151" s="10" t="s">
@@ -13406,7 +13560,7 @@
       <c r="D152" s="40"/>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>실행 결과별 재계획</t>
+          <t>결과에 맞춰 계획 수정</t>
         </is>
       </c>
       <c r="F152" s="10" t="s">
@@ -13482,7 +13636,7 @@
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>현재 주제·최근 발화 반영</t>
+          <t>현재 주제·최근 대화 반영</t>
         </is>
       </c>
       <c r="F153" s="10" t="s">
@@ -13556,7 +13710,7 @@
       <c r="D154" s="40"/>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>원요청·핵심 대상 보존</t>
+          <t>처음 요청·핵심 유산 유지</t>
         </is>
       </c>
       <c r="F154" s="10" t="s">
@@ -13706,7 +13860,7 @@
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>대상·항목·허용 ID 검증</t>
+          <t>대상·항목·허용 자료 확인</t>
         </is>
       </c>
       <c r="F156" s="10" t="s">
@@ -13852,8 +14006,10 @@
       <c r="D158" s="9" t="s">
         <v>252</v>
       </c>
-      <c r="E158" s="7" t="s">
-        <v>253</v>
+      <c r="E158" s="7" t="inlineStr">
+        <is>
+          <t>단어 질문·역사 질문 구분</t>
+        </is>
       </c>
       <c r="F158" s="10" t="s">
         <v>21</v>
@@ -13926,8 +14082,10 @@
       <c r="D159" s="40" t="s">
         <v>254</v>
       </c>
-      <c r="E159" s="7" t="s">
-        <v>255</v>
+      <c r="E159" s="7" t="inlineStr">
+        <is>
+          <t>관심 있는 역사 주제 파악</t>
+        </is>
       </c>
       <c r="F159" s="10" t="s">
         <v>21</v>
@@ -13998,8 +14156,10 @@
         <v>106</v>
       </c>
       <c r="D160" s="40"/>
-      <c r="E160" s="7" t="s">
-        <v>256</v>
+      <c r="E160" s="7" t="inlineStr">
+        <is>
+          <t>사용자 대화 내용과 연결</t>
+        </is>
       </c>
       <c r="F160" s="10" t="s">
         <v>21</v>
@@ -14072,8 +14232,10 @@
       <c r="D161" s="40" t="s">
         <v>257</v>
       </c>
-      <c r="E161" s="7" t="s">
-        <v>258</v>
+      <c r="E161" s="7" t="inlineStr">
+        <is>
+          <t>대화에서 학습 목표 파악</t>
+        </is>
       </c>
       <c r="F161" s="10" t="s">
         <v>21</v>
@@ -14218,8 +14380,10 @@
       <c r="D163" s="40" t="s">
         <v>260</v>
       </c>
-      <c r="E163" s="7" t="s">
-        <v>261</v>
+      <c r="E163" s="7" t="inlineStr">
+        <is>
+          <t>현재 요청·거부 의사 반영</t>
+        </is>
       </c>
       <c r="F163" s="10" t="s">
         <v>21</v>
@@ -14366,7 +14530,7 @@
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>질문 초점·문체 조절</t>
+          <t>질문 핵심·설명 방식 조절</t>
         </is>
       </c>
       <c r="F165" s="10" t="s">
@@ -14438,8 +14602,10 @@
         <v>106</v>
       </c>
       <c r="D166" s="40"/>
-      <c r="E166" s="7" t="s">
-        <v>265</v>
+      <c r="E166" s="7" t="inlineStr">
+        <is>
+          <t>수준별 설명 자세함 조절</t>
+        </is>
       </c>
       <c r="F166" s="10" t="s">
         <v>21</v>
@@ -14514,7 +14680,7 @@
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>문장·숫자·불확실성 검사</t>
+          <t>문장·숫자·추정 표현 확인</t>
         </is>
       </c>
       <c r="F167" s="10" t="s">
@@ -14588,7 +14754,7 @@
       <c r="D168" s="40"/>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>문장·인용·질문 적합성</t>
+          <t>문장·출처·질문 관련성</t>
         </is>
       </c>
       <c r="F168" s="10" t="s">
@@ -14662,8 +14828,10 @@
       <c r="D169" s="9" t="s">
         <v>269</v>
       </c>
-      <c r="E169" s="7" t="s">
-        <v>270</v>
+      <c r="E169" s="7" t="inlineStr">
+        <is>
+          <t>한 개념을 직접 설명하기</t>
+        </is>
       </c>
       <c r="F169" s="10" t="s">
         <v>21</v>
@@ -14738,7 +14906,7 @@
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>이해 판단·활동 완료 분리</t>
+          <t>이해 여부·활동 완료 구분</t>
         </is>
       </c>
       <c r="F170" s="10" t="s">
@@ -14810,8 +14978,10 @@
         <v>106</v>
       </c>
       <c r="D171" s="40"/>
-      <c r="E171" s="7" t="s">
-        <v>273</v>
+      <c r="E171" s="7" t="inlineStr">
+        <is>
+          <t>근거 번호·인용 확인</t>
+        </is>
       </c>
       <c r="F171" s="10" t="s">
         <v>21</v>
@@ -14886,7 +15056,7 @@
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>답안·개념·출처 연결</t>
+          <t>답안·학습 개념·출처 연결</t>
         </is>
       </c>
       <c r="F172" s="10" t="s">
@@ -15184,8 +15354,10 @@
       <c r="D176" s="40" t="s">
         <v>280</v>
       </c>
-      <c r="E176" s="7" t="s">
-        <v>281</v>
+      <c r="E176" s="7" t="inlineStr">
+        <is>
+          <t>반복해서 잘못 이해한 내용</t>
+        </is>
       </c>
       <c r="F176" s="10" t="s">
         <v>21</v>
@@ -15258,7 +15430,7 @@
       <c r="D177" s="40"/>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>다른 질문·활동 전환</t>
+          <t>다른 질문·활동으로 전환</t>
         </is>
       </c>
       <c r="F177" s="10" t="s">
@@ -15332,8 +15504,10 @@
       <c r="D178" s="40" t="s">
         <v>283</v>
       </c>
-      <c r="E178" s="7" t="s">
-        <v>284</v>
+      <c r="E178" s="7" t="inlineStr">
+        <is>
+          <t>직접 설명한 내용 종합</t>
+        </is>
       </c>
       <c r="F178" s="10" t="s">
         <v>21</v>
@@ -15406,7 +15580,7 @@
       <c r="D179" s="40"/>
       <c r="E179" s="7" t="inlineStr">
         <is>
-          <t>다음 사례·심화 선택</t>
+          <t>다음 사례·더 깊이 배우기</t>
         </is>
       </c>
       <c r="F179" s="10" t="s">
@@ -15480,8 +15654,10 @@
       <c r="D180" s="40" t="s">
         <v>286</v>
       </c>
-      <c r="E180" s="7" t="s">
-        <v>287</v>
+      <c r="E180" s="7" t="inlineStr">
+        <is>
+          <t>학습 처리 중 중단하기</t>
+        </is>
       </c>
       <c r="F180" s="10" t="s">
         <v>21</v>
@@ -15628,8 +15804,10 @@
       <c r="D182" s="40" t="s">
         <v>289</v>
       </c>
-      <c r="E182" s="7" t="s">
-        <v>290</v>
+      <c r="E182" s="7" t="inlineStr">
+        <is>
+          <t>학습자 반대 의견 보관</t>
+        </is>
       </c>
       <c r="F182" s="10" t="s">
         <v>21</v>
@@ -15700,8 +15878,10 @@
         <v>106</v>
       </c>
       <c r="D183" s="40"/>
-      <c r="E183" s="7" t="s">
-        <v>291</v>
+      <c r="E183" s="7" t="inlineStr">
+        <is>
+          <t>이해 판단 수정·심화 제외</t>
+        </is>
       </c>
       <c r="F183" s="10" t="s">
         <v>21</v>
@@ -15776,7 +15956,7 @@
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>부분 실패·기본 풀이 안내</t>
+          <t>일부 실패·기본 설명 안내</t>
         </is>
       </c>
       <c r="F184" s="10" t="s">
@@ -15924,8 +16104,10 @@
       <c r="D186" s="40" t="s">
         <v>295</v>
       </c>
-      <c r="E186" s="7" t="s">
-        <v>296</v>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>동시 처리·반복 횟수 제한</t>
+        </is>
       </c>
       <c r="F186" s="10" t="s">
         <v>21</v>
@@ -15996,8 +16178,10 @@
         <v>106</v>
       </c>
       <c r="D187" s="40"/>
-      <c r="E187" s="7" t="s">
-        <v>297</v>
+      <c r="E187" s="7" t="inlineStr">
+        <is>
+          <t>단계 수·대화 분량 제한</t>
+        </is>
       </c>
       <c r="F187" s="10" t="s">
         <v>21</v>
@@ -16070,8 +16254,10 @@
       <c r="D188" s="40" t="s">
         <v>298</v>
       </c>
-      <c r="E188" s="7" t="s">
-        <v>299</v>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>시대·구조의 근거 찾기</t>
+        </is>
       </c>
       <c r="F188" s="10" t="s">
         <v>21</v>
@@ -16142,8 +16328,10 @@
         <v>106</v>
       </c>
       <c r="D189" s="40"/>
-      <c r="E189" s="7" t="s">
-        <v>300</v>
+      <c r="E189" s="7" t="inlineStr">
+        <is>
+          <t>재료·종교 배경 찾기</t>
+        </is>
       </c>
       <c r="F189" s="10" t="s">
         <v>21</v>
@@ -16216,8 +16404,10 @@
       <c r="D190" s="40" t="s">
         <v>301</v>
       </c>
-      <c r="E190" s="7" t="s">
-        <v>302</v>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>처음 건립·재건 구분</t>
+        </is>
       </c>
       <c r="F190" s="10" t="s">
         <v>21</v>
@@ -16288,8 +16478,10 @@
         <v>106</v>
       </c>
       <c r="D191" s="40"/>
-      <c r="E191" s="7" t="s">
-        <v>303</v>
+      <c r="E191" s="7" t="inlineStr">
+        <is>
+          <t>추정 시기·주변 유산 구분</t>
+        </is>
       </c>
       <c r="F191" s="10" t="s">
         <v>21</v>
@@ -16362,8 +16554,10 @@
       <c r="D192" s="40" t="s">
         <v>304</v>
       </c>
-      <c r="E192" s="7" t="s">
-        <v>305</v>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>국내외 범위·유산 종류</t>
+        </is>
       </c>
       <c r="F192" s="10" t="s">
         <v>21</v>
@@ -16510,7 +16704,7 @@
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>검색어 변경·후보 재선택</t>
+          <t>검색어 바꾸기·후보 재선택</t>
         </is>
       </c>
       <c r="F194" s="10" t="s">
@@ -16582,8 +16776,10 @@
         <v>106</v>
       </c>
       <c r="D195" s="40"/>
-      <c r="E195" s="7" t="s">
-        <v>309</v>
+      <c r="E195" s="7" t="inlineStr">
+        <is>
+          <t>근거 부족 시 다음 안내</t>
+        </is>
       </c>
       <c r="F195" s="10" t="s">
         <v>21</v>
@@ -16658,7 +16854,7 @@
       </c>
       <c r="E196" s="7" t="inlineStr">
         <is>
-          <t>기준 대상·항목 비교</t>
+          <t>기준 유산·학습 항목 비교</t>
         </is>
       </c>
       <c r="F196" s="10" t="s">
@@ -16882,7 +17078,7 @@
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>저장 근거·질문 의미 검토</t>
+          <t>저장 자료·질문 뜻 확인</t>
         </is>
       </c>
       <c r="F199" s="10" t="s">
@@ -16954,8 +17150,10 @@
         <v>106</v>
       </c>
       <c r="D200" s="40"/>
-      <c r="E200" s="7" t="s">
-        <v>317</v>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>주장·인용의 근거 판단</t>
+        </is>
       </c>
       <c r="F200" s="10" t="s">
         <v>21</v>
@@ -17178,7 +17376,7 @@
       </c>
       <c r="E203" s="7" t="inlineStr">
         <is>
-          <t>현재 목표의 퀴즈 생성</t>
+          <t>현재 목표에 맞는 퀴즈</t>
         </is>
       </c>
       <c r="F203" s="10" t="s">
@@ -17324,8 +17522,10 @@
       <c r="D205" s="9" t="s">
         <v>324</v>
       </c>
-      <c r="E205" s="7" t="s">
-        <v>325</v>
+      <c r="E205" s="7" t="inlineStr">
+        <is>
+          <t>확인한 자료로 기본 문제</t>
+        </is>
       </c>
       <c r="F205" s="10" t="s">
         <v>21</v>
@@ -17398,8 +17598,10 @@
       <c r="D206" s="40" t="s">
         <v>326</v>
       </c>
-      <c r="E206" s="7" t="s">
-        <v>327</v>
+      <c r="E206" s="7" t="inlineStr">
+        <is>
+          <t>답안 채점·점수 계산</t>
+        </is>
       </c>
       <c r="F206" s="10" t="s">
         <v>21</v>
@@ -17470,8 +17672,10 @@
         <v>106</v>
       </c>
       <c r="D207" s="40"/>
-      <c r="E207" s="7" t="s">
-        <v>328</v>
+      <c r="E207" s="7" t="inlineStr">
+        <is>
+          <t>문제별 해설·근거 연결</t>
+        </is>
       </c>
       <c r="F207" s="10" t="s">
         <v>21</v>
@@ -17546,7 +17750,7 @@
       </c>
       <c r="E208" s="7" t="inlineStr">
         <is>
-          <t>현재 비교·오답 근거 조회</t>
+          <t>현재 비교·오답 근거 찾기</t>
         </is>
       </c>
       <c r="F208" s="10" t="s">
@@ -17766,8 +17970,10 @@
         <v>106</v>
       </c>
       <c r="D211" s="40"/>
-      <c r="E211" s="7" t="s">
-        <v>334</v>
+      <c r="E211" s="7" t="inlineStr">
+        <is>
+          <t>주제 바꾸기·판단 수정</t>
+        </is>
       </c>
       <c r="F211" s="10" t="s">
         <v>21</v>
@@ -17840,8 +18046,10 @@
       <c r="D212" s="40" t="s">
         <v>335</v>
       </c>
-      <c r="E212" s="7" t="s">
-        <v>336</v>
+      <c r="E212" s="7" t="inlineStr">
+        <is>
+          <t>사용자·비교 수정본 저장</t>
+        </is>
       </c>
       <c r="F212" s="10" t="s">
         <v>21</v>
@@ -17914,7 +18122,7 @@
       <c r="D213" s="40"/>
       <c r="E213" s="7" t="inlineStr">
         <is>
-          <t>비교·퀴즈 재사용·재탐구</t>
+          <t>비교·퀴즈 활용·다시 탐구</t>
         </is>
       </c>
       <c r="F213" s="10" t="s">
@@ -17988,8 +18196,10 @@
       <c r="D214" s="40" t="s">
         <v>338</v>
       </c>
-      <c r="E214" s="7" t="s">
-        <v>339</v>
+      <c r="E214" s="7" t="inlineStr">
+        <is>
+          <t>비교·출처 담은 활동지</t>
+        </is>
       </c>
       <c r="F214" s="10" t="s">
         <v>21</v>
@@ -18286,7 +18496,7 @@
       </c>
       <c r="E218" s="7" t="inlineStr">
         <is>
-          <t>대상 보존·재계획 검증</t>
+          <t>기준 유산 유지·계획 수정</t>
         </is>
       </c>
       <c r="F218" s="10" t="s">
@@ -18506,8 +18716,10 @@
         <v>18</v>
       </c>
       <c r="D221" s="40"/>
-      <c r="E221" s="7" t="s">
-        <v>350</v>
+      <c r="E221" s="7" t="inlineStr">
+        <is>
+          <t>관심 파악·새로고침 유지</t>
+        </is>
       </c>
       <c r="F221" s="10" t="s">
         <v>21</v>
@@ -18582,7 +18794,7 @@
       </c>
       <c r="E222" s="7" t="inlineStr">
         <is>
-          <t>중단·정정·주제 혼입 차단</t>
+          <t>중단·정정·다른 주제 구분</t>
         </is>
       </c>
       <c r="F222" s="10" t="s">
@@ -18728,8 +18940,10 @@
       <c r="D224" s="40" t="s">
         <v>354</v>
       </c>
-      <c r="E224" s="7" t="s">
-        <v>355</v>
+      <c r="E224" s="7" t="inlineStr">
+        <is>
+          <t>다른 사람 대화·설정 차단</t>
+        </is>
       </c>
       <c r="F224" s="10" t="s">
         <v>21</v>
@@ -18800,8 +19014,10 @@
         <v>18</v>
       </c>
       <c r="D225" s="40"/>
-      <c r="E225" s="7" t="s">
-        <v>356</v>
+      <c r="E225" s="7" t="inlineStr">
+        <is>
+          <t>다른 사람 기록·복습 차단</t>
+        </is>
       </c>
       <c r="F225" s="10" t="s">
         <v>21</v>
@@ -18874,8 +19090,10 @@
       <c r="D226" s="40" t="s">
         <v>357</v>
       </c>
-      <c r="E226" s="7" t="s">
-        <v>358</v>
+      <c r="E226" s="7" t="inlineStr">
+        <is>
+          <t>원문 유지·자료 이용 제한</t>
+        </is>
       </c>
       <c r="F226" s="10" t="s">
         <v>21</v>
@@ -19022,7 +19240,7 @@
       </c>
       <c r="E228" s="7" t="inlineStr">
         <is>
-          <t>전체777개 회귀 검사</t>
+          <t>기존 기능796개 재검사</t>
         </is>
       </c>
       <c r="F228" s="10" t="s">
@@ -19096,7 +19314,7 @@
       <c r="D229" s="40"/>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>2환경·관련45개 회귀</t>
+          <t>두 환경·관련61개 재검사</t>
         </is>
       </c>
       <c r="F229" s="10" t="s">
@@ -19172,7 +19390,7 @@
       </c>
       <c r="E230" s="7" t="inlineStr">
         <is>
-          <t>실제 관심사·목표 검증</t>
+          <t>실제 관심사·목표 파악 확인</t>
         </is>
       </c>
       <c r="F230" s="10" t="s">
@@ -19248,7 +19466,7 @@
       <c r="D231" s="40"/>
       <c r="E231" s="7" t="inlineStr">
         <is>
-          <t>실제 목표 변경·교정 검증</t>
+          <t>실제 목표 변경·수정 확인</t>
         </is>
       </c>
       <c r="F231" s="10" t="s">
@@ -19326,7 +19544,7 @@
       </c>
       <c r="E232" s="7" t="inlineStr">
         <is>
-          <t>실제 답변·원문 근거 검토</t>
+          <t>실제 답변·원문 근거 확인</t>
         </is>
       </c>
       <c r="F232" s="10" t="s">
@@ -19402,7 +19620,7 @@
       <c r="D233" s="40"/>
       <c r="E233" s="7" t="inlineStr">
         <is>
-          <t>실제 난도·질문 적합성</t>
+          <t>실제 난도·질문 관련성</t>
         </is>
       </c>
       <c r="F233" s="10" t="s">
@@ -19480,7 +19698,7 @@
       </c>
       <c r="E234" s="7" t="inlineStr">
         <is>
-          <t>실제 정답·오개념 판단</t>
+          <t>실제 정답·잘못 이해한 답</t>
         </is>
       </c>
       <c r="F234" s="10" t="s">
@@ -19556,7 +19774,7 @@
       <c r="D235" s="40"/>
       <c r="E235" s="7" t="inlineStr">
         <is>
-          <t>실제 보충·심화 분기</t>
+          <t>실제 보충·심화 선택 확인</t>
         </is>
       </c>
       <c r="F235" s="10" t="s">
@@ -19632,8 +19850,10 @@
       <c r="D236" s="40" t="s">
         <v>372</v>
       </c>
-      <c r="E236" s="7" t="s">
-        <v>373</v>
+      <c r="E236" s="7" t="inlineStr">
+        <is>
+          <t>한국어 이름·시기 확인</t>
+        </is>
       </c>
       <c r="F236" s="10" t="s">
         <v>21</v>
@@ -19704,8 +19924,10 @@
         <v>18</v>
       </c>
       <c r="D237" s="40"/>
-      <c r="E237" s="7" t="s">
-        <v>374</v>
+      <c r="E237" s="7" t="inlineStr">
+        <is>
+          <t>설명 대상·풀이 대조</t>
+        </is>
       </c>
       <c r="F237" s="10" t="s">
         <v>21</v>
@@ -19780,7 +20002,7 @@
       </c>
       <c r="E238" s="7" t="inlineStr">
         <is>
-          <t>코스별45회 모의 흐름</t>
+          <t>코스별45회 학습 예행연습</t>
         </is>
       </c>
       <c r="F238" s="10" t="s">
@@ -20000,8 +20222,10 @@
         <v>18</v>
       </c>
       <c r="D241" s="40"/>
-      <c r="E241" s="7" t="s">
-        <v>380</v>
+      <c r="E241" s="7" t="inlineStr">
+        <is>
+          <t>마이크 허용·거부·재허용</t>
+        </is>
       </c>
       <c r="F241" s="10" t="s">
         <v>21</v>
@@ -20074,8 +20298,10 @@
       <c r="D242" s="40" t="s">
         <v>381</v>
       </c>
-      <c r="E242" s="7" t="s">
-        <v>382</v>
+      <c r="E242" s="7" t="inlineStr">
+        <is>
+          <t>휴대전화 앱 추가·재실행</t>
+        </is>
       </c>
       <c r="F242" s="10" t="s">
         <v>21</v>
@@ -20146,8 +20372,10 @@
         <v>18</v>
       </c>
       <c r="D243" s="40"/>
-      <c r="E243" s="7" t="s">
-        <v>383</v>
+      <c r="E243" s="7" t="inlineStr">
+        <is>
+          <t>업데이트·연결 끊김</t>
+        </is>
       </c>
       <c r="F243" s="10" t="s">
         <v>21</v>
@@ -20222,7 +20450,7 @@
       </c>
       <c r="E244" s="7" t="inlineStr">
         <is>
-          <t>키보드 확인·실제 확대 대기</t>
+          <t>키보드 확인·확대 점검 대기</t>
         </is>
       </c>
       <c r="F244" s="10" t="s">
@@ -20296,7 +20524,7 @@
       <c r="D245" s="40"/>
       <c r="E245" s="7" t="inlineStr">
         <is>
-          <t>체험 초기화·기록 분리</t>
+          <t>5분 초기화·이전 기록 차단</t>
         </is>
       </c>
       <c r="F245" s="10" t="s">
@@ -20594,7 +20822,7 @@
       <c r="D249" s="40"/>
       <c r="E249" s="7" t="inlineStr">
         <is>
-          <t>실제 완주·복구·시간·비용</t>
+          <t>실제 완료·복구·시간·비용</t>
         </is>
       </c>
       <c r="F249" s="10" t="s">
@@ -20672,8 +20900,10 @@
       <c r="D250" s="40" t="s">
         <v>396</v>
       </c>
-      <c r="E250" s="7" t="s">
-        <v>397</v>
+      <c r="E250" s="7" t="inlineStr">
+        <is>
+          <t>필요한 도구·PC 실행 정리</t>
+        </is>
       </c>
       <c r="F250" s="10" t="s">
         <v>21</v>
@@ -20744,8 +20974,10 @@
         <v>395</v>
       </c>
       <c r="D251" s="40"/>
-      <c r="E251" s="7" t="s">
-        <v>398</v>
+      <c r="E251" s="7" t="inlineStr">
+        <is>
+          <t>API 키 공개하지 않기</t>
+        </is>
       </c>
       <c r="F251" s="10" t="s">
         <v>21</v>
@@ -21114,7 +21346,7 @@
       </c>
       <c r="E256" s="7" t="inlineStr">
         <is>
-          <t>복제·환경 완료·키 대기</t>
+          <t>내려받기·설치 완료·키 대기</t>
         </is>
       </c>
       <c r="F256" s="10" t="s">
@@ -21264,8 +21496,10 @@
       <c r="D258" s="40" t="s">
         <v>408</v>
       </c>
-      <c r="E258" s="7" t="s">
-        <v>409</v>
+      <c r="E258" s="7" t="inlineStr">
+        <is>
+          <t>설치·학습 순서 안내</t>
+        </is>
       </c>
       <c r="F258" s="10" t="s">
         <v>21</v>
@@ -21338,7 +21572,7 @@
       <c r="D259" s="40"/>
       <c r="E259" s="7" t="inlineStr">
         <is>
-          <t>Agent 역할·지원 범위 안내</t>
+          <t>AI Agent 역할·범위 안내</t>
         </is>
       </c>
       <c r="F259" s="10" t="s">
@@ -21414,7 +21648,7 @@
       </c>
       <c r="E260" s="7" t="inlineStr">
         <is>
-          <t>코드·검증 문서 반영</t>
+          <t>코드·점검 문서 올리기</t>
         </is>
       </c>
       <c r="F260" s="10" t="s">
@@ -21492,7 +21726,7 @@
       </c>
       <c r="E261" s="7" t="inlineStr">
         <is>
-          <t>구현·측정 범위 정리</t>
+          <t>구현한 기능·측정 범위</t>
         </is>
       </c>
       <c r="F261" s="10" t="s">
@@ -21566,7 +21800,7 @@
       <c r="D262" s="40"/>
       <c r="E262" s="7" t="inlineStr">
         <is>
-          <t>미측정·기기·교육 한계</t>
+          <t>미측정·기기·수업의 한계</t>
         </is>
       </c>
       <c r="F262" s="10" t="s">
@@ -21640,8 +21874,10 @@
       <c r="D263" s="40" t="s">
         <v>417</v>
       </c>
-      <c r="E263" s="7" t="s">
-        <v>418</v>
+      <c r="E263" s="7" t="inlineStr">
+        <is>
+          <t>설계·개발·점검 결과 작성</t>
+        </is>
       </c>
       <c r="F263" s="10" t="s">
         <v>21</v>
@@ -21786,8 +22022,10 @@
       <c r="D265" s="40" t="s">
         <v>420</v>
       </c>
-      <c r="E265" s="7" t="s">
-        <v>421</v>
+      <c r="E265" s="7" t="inlineStr">
+        <is>
+          <t>목적·AI Agent·화면 구성</t>
+        </is>
       </c>
       <c r="F265" s="10" t="s">
         <v>21</v>
@@ -21858,8 +22096,10 @@
         <v>18</v>
       </c>
       <c r="D266" s="40"/>
-      <c r="E266" s="7" t="s">
-        <v>422</v>
+      <c r="E266" s="7" t="inlineStr">
+        <is>
+          <t>점검 결과 발표 구성</t>
+        </is>
       </c>
       <c r="F266" s="10" t="s">
         <v>21</v>
@@ -22004,8 +22244,10 @@
         <v>18</v>
       </c>
       <c r="D268" s="40"/>
-      <c r="E268" s="7" t="s">
-        <v>425</v>
+      <c r="E268" s="7" t="inlineStr">
+        <is>
+          <t>오류·자료 부족 시 예비 시연</t>
+        </is>
       </c>
       <c r="F268" s="10" t="s">
         <v>21</v>
@@ -22152,8 +22394,10 @@
         <v>18</v>
       </c>
       <c r="D270" s="40"/>
-      <c r="E270" s="7" t="s">
-        <v>428</v>
+      <c r="E270" s="7" t="inlineStr">
+        <is>
+          <t>코드·비밀정보 제외·제출</t>
+        </is>
       </c>
       <c r="F270" s="10" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Add glossary support after live dialogue check and record quota-limited results
</commit_message>
<xml_diff>
--- a/docs/CultureBridge_WBS_실제현황_2026-10-25.xlsx
+++ b/docs/CultureBridge_WBS_실제현황_2026-10-25.xlsx
@@ -19240,7 +19240,7 @@
       </c>
       <c r="E228" s="7" t="inlineStr">
         <is>
-          <t>기존 기능796개 재검사</t>
+          <t>기존 기능801개 재검사</t>
         </is>
       </c>
       <c r="F228" s="10" t="s">
@@ -19314,7 +19314,7 @@
       <c r="D229" s="40"/>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>두 환경·관련61개 재검사</t>
+          <t>두 환경·관련66개 재검사</t>
         </is>
       </c>
       <c r="F229" s="10" t="s">

</xml_diff>

<commit_message>
Improve easy explanations and history relevance; distinguish review lookup from completion
</commit_message>
<xml_diff>
--- a/docs/CultureBridge_WBS_실제현황_2026-10-25.xlsx
+++ b/docs/CultureBridge_WBS_실제현황_2026-10-25.xlsx
@@ -19240,7 +19240,7 @@
       </c>
       <c r="E228" s="7" t="inlineStr">
         <is>
-          <t>기존 기능801개 재검사</t>
+          <t>기존 기능815개 재검사</t>
         </is>
       </c>
       <c r="F228" s="10" t="s">
@@ -19314,7 +19314,7 @@
       <c r="D229" s="40"/>
       <c r="E229" s="7" t="inlineStr">
         <is>
-          <t>두 환경·관련66개 재검사</t>
+          <t>두 환경·관련91개 재검사</t>
         </is>
       </c>
       <c r="F229" s="10" t="s">

</xml_diff>